<commit_message>
MROY catalog updates, cleanup scripts, table creation fix
</commit_message>
<xml_diff>
--- a/app/database/MRA11/mroy_MRA1_13_Temperature_Extended_Options.xlsx
+++ b/app/database/MRA11/mroy_MRA1_13_Temperature_Extended_Options.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8190" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="Temperature_Extended_Options" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Temperature_Extended_Options" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -22,60 +21,59 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
-    <t xml:space="preserve">code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">price_usd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">consult_factory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">requires_lube_option_5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">metallic_only</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standard: Ambient -20°F to 120°F (29°C to 49°C); Liquid -20°F to 200°F (-29°C to 93°C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low ambient: Ambient -40°F to 120°F (-40°C to 49°C); Liquid -45°F to 200°F (-43°C to 93°C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Must select lubrication option 5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High temperature (includes PEEK diaphragm): Ambient 20°F to 120°F (-6°C to 49°C); Liquid 50°F to 300°F (10°C to 149°C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metallic liquid ends only.</t>
+    <t>code</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>price_usd</t>
+  </si>
+  <si>
+    <t>consult_factory</t>
+  </si>
+  <si>
+    <t>requires_lube_option_5</t>
+  </si>
+  <si>
+    <t>metallic_only</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>Standard: Ambient -20°F to 120°F (29°C to 49°C); Liquid -20°F to 200°F (-29°C to 93°C)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Low ambient: Ambient -40°F to 120°F (-40°C to 49°C); Liquid -45°F to 200°F (-43°C to 93°C)</t>
+  </si>
+  <si>
+    <t>Must select lubrication option 5.</t>
+  </si>
+  <si>
+    <t>High temperature (includes PEEK diaphragm): Ambient 20°F to 120°F (-6°C to 49°C); Liquid 50°F to 300°F (10°C to 149°C)</t>
+  </si>
+  <si>
+    <t>Metallic liquid ends only.</t>
+  </si>
+  <si>
+    <t>NULL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,22 +82,7 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -116,7 +99,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -124,104 +107,70 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -229,12 +178,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -263,7 +212,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -284,7 +233,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -335,7 +284,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -353,33 +302,32 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:J1048576"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="103.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="28.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="1" width="10.16"/>
+    <col min="1" max="1" width="5.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="104" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12.140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="28.5703125" style="1" customWidth="1"/>
+    <col min="8" max="10" width="10.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -405,14 +353,14 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" s="4">
         <v>0</v>
       </c>
       <c r="D2" s="5" t="b">
@@ -428,15 +376,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D3" s="5" t="b">
         <v>1</v>
@@ -448,17 +396,17 @@
         <v>0</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="4">
         <v>903</v>
       </c>
       <c r="D4" s="5" t="b">
@@ -471,74 +419,62 @@
         <v>1</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="C5" s="4"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="C6" s="4"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
     </row>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>